<commit_message>
added compliance map in pci single dss
</commit_message>
<xml_diff>
--- a/Audit_Code/public/PCI_DSS_4_Single_TSP.xlsx
+++ b/Audit_Code/public/PCI_DSS_4_Single_TSP.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ab\Desktop\Compliance\Audit_Code\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muhammad.abdullah\Documents\Compliance\Audit_Code\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9630"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9636"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="581">
   <si>
     <t>Requirement</t>
   </si>
@@ -2216,6 +2216,9 @@
   </si>
   <si>
     <t>All service providers with existing connection points to POS POI terminals that use SSL and/or early TLS as defined in A2.1, provide a secure service offering.</t>
+  </si>
+  <si>
+    <t>Unknown</t>
   </si>
 </sst>
 </file>
@@ -2589,17 +2592,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G257"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" customWidth="1"/>
+    <col min="5" max="5" width="16.109375" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" customWidth="1"/>
     <col min="7" max="7" width="0" hidden="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" hidden="1"/>
+    <col min="8" max="16384" width="9.109375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2611,7 +2614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -2629,7 +2632,7 @@
       </c>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" ht="280.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -2647,7 +2650,7 @@
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>1</v>
       </c>
@@ -2665,7 +2668,7 @@
       </c>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>1</v>
       </c>
@@ -2683,7 +2686,7 @@
       </c>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -2701,7 +2704,7 @@
       </c>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>1</v>
       </c>
@@ -2719,7 +2722,7 @@
       </c>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>1</v>
       </c>
@@ -2737,7 +2740,7 @@
       </c>
       <c r="F8" s="5"/>
     </row>
-    <row r="9" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>1</v>
       </c>
@@ -2755,7 +2758,7 @@
       </c>
       <c r="F9" s="5"/>
     </row>
-    <row r="10" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>1</v>
       </c>
@@ -2773,7 +2776,7 @@
       </c>
       <c r="F10" s="5"/>
     </row>
-    <row r="11" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>1</v>
       </c>
@@ -2791,7 +2794,7 @@
       </c>
       <c r="F11" s="5"/>
     </row>
-    <row r="12" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>1</v>
       </c>
@@ -2809,7 +2812,7 @@
       </c>
       <c r="F12" s="5"/>
     </row>
-    <row r="13" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>1</v>
       </c>
@@ -2827,7 +2830,7 @@
       </c>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>1</v>
       </c>
@@ -2845,7 +2848,7 @@
       </c>
       <c r="F14" s="5"/>
     </row>
-    <row r="15" spans="1:6" ht="267.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="277.2" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>1</v>
       </c>
@@ -2863,7 +2866,7 @@
       </c>
       <c r="F15" s="5"/>
     </row>
-    <row r="16" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>1</v>
       </c>
@@ -2881,7 +2884,7 @@
       </c>
       <c r="F16" s="5"/>
     </row>
-    <row r="17" spans="1:6" ht="318.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="303.60000000000002" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>1</v>
       </c>
@@ -2899,7 +2902,7 @@
       </c>
       <c r="F17" s="5"/>
     </row>
-    <row r="18" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>1</v>
       </c>
@@ -2917,7 +2920,7 @@
       </c>
       <c r="F18" s="5"/>
     </row>
-    <row r="19" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>1</v>
       </c>
@@ -2935,7 +2938,7 @@
       </c>
       <c r="F19" s="5"/>
     </row>
-    <row r="20" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>1</v>
       </c>
@@ -2953,7 +2956,7 @@
       </c>
       <c r="F20" s="5"/>
     </row>
-    <row r="21" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>1</v>
       </c>
@@ -2971,7 +2974,7 @@
       </c>
       <c r="F21" s="5"/>
     </row>
-    <row r="22" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="198" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>2</v>
       </c>
@@ -2989,7 +2992,7 @@
       </c>
       <c r="F22" s="5"/>
     </row>
-    <row r="23" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="198" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
         <v>2</v>
       </c>
@@ -3007,7 +3010,7 @@
       </c>
       <c r="F23" s="5"/>
     </row>
-    <row r="24" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>2</v>
       </c>
@@ -3025,7 +3028,7 @@
       </c>
       <c r="F24" s="5"/>
     </row>
-    <row r="25" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
         <v>2</v>
       </c>
@@ -3043,7 +3046,7 @@
       </c>
       <c r="F25" s="5"/>
     </row>
-    <row r="26" spans="1:6" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>2</v>
       </c>
@@ -3061,7 +3064,7 @@
       </c>
       <c r="F26" s="5"/>
     </row>
-    <row r="27" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="409.2" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>2</v>
       </c>
@@ -3079,7 +3082,7 @@
       </c>
       <c r="F27" s="5"/>
     </row>
-    <row r="28" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>2</v>
       </c>
@@ -3097,7 +3100,7 @@
       </c>
       <c r="F28" s="5"/>
     </row>
-    <row r="29" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="237.6" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
         <v>2</v>
       </c>
@@ -3115,7 +3118,7 @@
       </c>
       <c r="F29" s="5"/>
     </row>
-    <row r="30" spans="1:6" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>2</v>
       </c>
@@ -3133,7 +3136,7 @@
       </c>
       <c r="F30" s="5"/>
     </row>
-    <row r="31" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
         <v>2</v>
       </c>
@@ -3151,7 +3154,7 @@
       </c>
       <c r="F31" s="5"/>
     </row>
-    <row r="32" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>3</v>
       </c>
@@ -3169,7 +3172,7 @@
       </c>
       <c r="F32" s="5"/>
     </row>
-    <row r="33" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>3</v>
       </c>
@@ -3187,7 +3190,7 @@
       </c>
       <c r="F33" s="5"/>
     </row>
-    <row r="34" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>3</v>
       </c>
@@ -3205,7 +3208,7 @@
       </c>
       <c r="F34" s="5"/>
     </row>
-    <row r="35" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
         <v>3</v>
       </c>
@@ -3225,7 +3228,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>3</v>
       </c>
@@ -3243,7 +3246,7 @@
       </c>
       <c r="F36" s="5"/>
     </row>
-    <row r="37" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A37" s="4">
         <v>3</v>
       </c>
@@ -3261,7 +3264,7 @@
       </c>
       <c r="F37" s="5"/>
     </row>
-    <row r="38" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>3</v>
       </c>
@@ -3279,7 +3282,7 @@
       </c>
       <c r="F38" s="5"/>
     </row>
-    <row r="39" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
         <v>3</v>
       </c>
@@ -3297,7 +3300,7 @@
       </c>
       <c r="F39" s="5"/>
     </row>
-    <row r="40" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>3</v>
       </c>
@@ -3317,7 +3320,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A41" s="4">
         <v>3</v>
       </c>
@@ -3335,7 +3338,7 @@
       </c>
       <c r="F41" s="5"/>
     </row>
-    <row r="42" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>3</v>
       </c>
@@ -3355,7 +3358,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A43" s="4">
         <v>3</v>
       </c>
@@ -3373,7 +3376,7 @@
       </c>
       <c r="F43" s="5"/>
     </row>
-    <row r="44" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>3</v>
       </c>
@@ -3393,7 +3396,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A45" s="4">
         <v>3</v>
       </c>
@@ -3411,7 +3414,7 @@
       </c>
       <c r="F45" s="5"/>
     </row>
-    <row r="46" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A46" s="4">
         <v>3</v>
       </c>
@@ -3431,7 +3434,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="318.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" ht="330" x14ac:dyDescent="0.3">
       <c r="A47" s="4">
         <v>3</v>
       </c>
@@ -3451,7 +3454,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A48" s="4">
         <v>3</v>
       </c>
@@ -3469,7 +3472,7 @@
       </c>
       <c r="F48" s="5"/>
     </row>
-    <row r="49" spans="1:6" ht="408" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A49" s="4">
         <v>3</v>
       </c>
@@ -3487,7 +3490,7 @@
       </c>
       <c r="F49" s="5"/>
     </row>
-    <row r="50" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
         <v>3</v>
       </c>
@@ -3505,7 +3508,7 @@
       </c>
       <c r="F50" s="5"/>
     </row>
-    <row r="51" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
         <v>3</v>
       </c>
@@ -3525,7 +3528,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A52" s="4">
         <v>3</v>
       </c>
@@ -3543,7 +3546,7 @@
       </c>
       <c r="F52" s="5"/>
     </row>
-    <row r="53" spans="1:6" ht="102" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A53" s="4">
         <v>3</v>
       </c>
@@ -3561,7 +3564,7 @@
       </c>
       <c r="F53" s="5"/>
     </row>
-    <row r="54" spans="1:6" ht="102" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A54" s="4">
         <v>3</v>
       </c>
@@ -3579,7 +3582,7 @@
       </c>
       <c r="F54" s="5"/>
     </row>
-    <row r="55" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A55" s="4">
         <v>3</v>
       </c>
@@ -3597,7 +3600,7 @@
       </c>
       <c r="F55" s="5"/>
     </row>
-    <row r="56" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A56" s="4">
         <v>3</v>
       </c>
@@ -3615,7 +3618,7 @@
       </c>
       <c r="F56" s="5"/>
     </row>
-    <row r="57" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A57" s="4">
         <v>3</v>
       </c>
@@ -3633,7 +3636,7 @@
       </c>
       <c r="F57" s="5"/>
     </row>
-    <row r="58" spans="1:6" ht="357" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" ht="369.6" x14ac:dyDescent="0.3">
       <c r="A58" s="4">
         <v>3</v>
       </c>
@@ -3651,7 +3654,7 @@
       </c>
       <c r="F58" s="5"/>
     </row>
-    <row r="59" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A59" s="4">
         <v>3</v>
       </c>
@@ -3669,7 +3672,7 @@
       </c>
       <c r="F59" s="5"/>
     </row>
-    <row r="60" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A60" s="4">
         <v>3</v>
       </c>
@@ -3687,7 +3690,7 @@
       </c>
       <c r="F60" s="5"/>
     </row>
-    <row r="61" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A61" s="4">
         <v>3</v>
       </c>
@@ -3705,7 +3708,7 @@
       </c>
       <c r="F61" s="5"/>
     </row>
-    <row r="62" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A62" s="4">
         <v>3</v>
       </c>
@@ -3723,7 +3726,7 @@
       </c>
       <c r="F62" s="5"/>
     </row>
-    <row r="63" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A63" s="4">
         <v>3</v>
       </c>
@@ -3741,7 +3744,7 @@
       </c>
       <c r="F63" s="5"/>
     </row>
-    <row r="64" spans="1:6" ht="280.5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" ht="290.39999999999998" x14ac:dyDescent="0.3">
       <c r="A64" s="4">
         <v>4</v>
       </c>
@@ -3759,7 +3762,7 @@
       </c>
       <c r="F64" s="5"/>
     </row>
-    <row r="65" spans="1:6" ht="280.5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" ht="290.39999999999998" x14ac:dyDescent="0.3">
       <c r="A65" s="4">
         <v>4</v>
       </c>
@@ -3777,7 +3780,7 @@
       </c>
       <c r="F65" s="5"/>
     </row>
-    <row r="66" spans="1:6" ht="408" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A66" s="4">
         <v>4</v>
       </c>
@@ -3795,7 +3798,7 @@
       </c>
       <c r="F66" s="5"/>
     </row>
-    <row r="67" spans="1:6" ht="255" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" ht="264" x14ac:dyDescent="0.3">
       <c r="A67" s="4">
         <v>4</v>
       </c>
@@ -3815,7 +3818,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A68" s="4">
         <v>4</v>
       </c>
@@ -3835,7 +3838,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A69" s="4">
         <v>4</v>
       </c>
@@ -3853,7 +3856,7 @@
       </c>
       <c r="F69" s="5"/>
     </row>
-    <row r="70" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A70" s="4">
         <v>4</v>
       </c>
@@ -3871,7 +3874,7 @@
       </c>
       <c r="F70" s="5"/>
     </row>
-    <row r="71" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A71" s="4">
         <v>5</v>
       </c>
@@ -3889,7 +3892,7 @@
       </c>
       <c r="F71" s="5"/>
     </row>
-    <row r="72" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A72" s="4">
         <v>5</v>
       </c>
@@ -3907,7 +3910,7 @@
       </c>
       <c r="F72" s="5"/>
     </row>
-    <row r="73" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A73" s="4">
         <v>5</v>
       </c>
@@ -3925,7 +3928,7 @@
       </c>
       <c r="F73" s="5"/>
     </row>
-    <row r="74" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A74" s="4">
         <v>5</v>
       </c>
@@ -3943,7 +3946,7 @@
       </c>
       <c r="F74" s="5"/>
     </row>
-    <row r="75" spans="1:6" ht="344.25" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" ht="343.2" x14ac:dyDescent="0.3">
       <c r="A75" s="4">
         <v>5</v>
       </c>
@@ -3961,7 +3964,7 @@
       </c>
       <c r="F75" s="5"/>
     </row>
-    <row r="76" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A76" s="4">
         <v>5</v>
       </c>
@@ -3981,7 +3984,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A77" s="4">
         <v>5</v>
       </c>
@@ -3999,7 +4002,7 @@
       </c>
       <c r="F77" s="5"/>
     </row>
-    <row r="78" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A78" s="4">
         <v>5</v>
       </c>
@@ -4017,7 +4020,7 @@
       </c>
       <c r="F78" s="5"/>
     </row>
-    <row r="79" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" ht="198" x14ac:dyDescent="0.3">
       <c r="A79" s="4">
         <v>5</v>
       </c>
@@ -4037,7 +4040,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="267.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" ht="277.2" x14ac:dyDescent="0.3">
       <c r="A80" s="4">
         <v>5</v>
       </c>
@@ -4057,7 +4060,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A81" s="4">
         <v>5</v>
       </c>
@@ -4075,7 +4078,7 @@
       </c>
       <c r="F81" s="5"/>
     </row>
-    <row r="82" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A82" s="4">
         <v>5</v>
       </c>
@@ -4093,7 +4096,7 @@
       </c>
       <c r="F82" s="5"/>
     </row>
-    <row r="83" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A83" s="4">
         <v>5</v>
       </c>
@@ -4113,7 +4116,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A84" s="4">
         <v>6</v>
       </c>
@@ -4131,7 +4134,7 @@
       </c>
       <c r="F84" s="5"/>
     </row>
-    <row r="85" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A85" s="4">
         <v>6</v>
       </c>
@@ -4149,7 +4152,7 @@
       </c>
       <c r="F85" s="5"/>
     </row>
-    <row r="86" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A86" s="4">
         <v>6</v>
       </c>
@@ -4167,7 +4170,7 @@
       </c>
       <c r="F86" s="5"/>
     </row>
-    <row r="87" spans="1:6" ht="344.25" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" ht="343.2" x14ac:dyDescent="0.3">
       <c r="A87" s="4">
         <v>6</v>
       </c>
@@ -4185,7 +4188,7 @@
       </c>
       <c r="F87" s="5"/>
     </row>
-    <row r="88" spans="1:6" ht="331.5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" ht="343.2" x14ac:dyDescent="0.3">
       <c r="A88" s="4">
         <v>6</v>
       </c>
@@ -4203,7 +4206,7 @@
       </c>
       <c r="F88" s="5"/>
     </row>
-    <row r="89" spans="1:6" ht="293.25" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" ht="290.39999999999998" x14ac:dyDescent="0.3">
       <c r="A89" s="4">
         <v>6</v>
       </c>
@@ -4221,7 +4224,7 @@
       </c>
       <c r="F89" s="5"/>
     </row>
-    <row r="90" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A90" s="4">
         <v>6</v>
       </c>
@@ -4239,7 +4242,7 @@
       </c>
       <c r="F90" s="5"/>
     </row>
-    <row r="91" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A91" s="4">
         <v>6</v>
       </c>
@@ -4257,7 +4260,7 @@
       </c>
       <c r="F91" s="5"/>
     </row>
-    <row r="92" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A92" s="4">
         <v>6</v>
       </c>
@@ -4277,7 +4280,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A93" s="4">
         <v>6</v>
       </c>
@@ -4295,7 +4298,7 @@
       </c>
       <c r="F93" s="5"/>
     </row>
-    <row r="94" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A94" s="4">
         <v>6</v>
       </c>
@@ -4313,7 +4316,7 @@
       </c>
       <c r="F94" s="5"/>
     </row>
-    <row r="95" spans="1:6" ht="395.25" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" ht="382.8" x14ac:dyDescent="0.3">
       <c r="A95" s="4">
         <v>6</v>
       </c>
@@ -4333,7 +4336,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="96" spans="1:6" ht="318.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A96" s="4">
         <v>6</v>
       </c>
@@ -4353,7 +4356,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A97" s="4">
         <v>6</v>
       </c>
@@ -4371,7 +4374,7 @@
       </c>
       <c r="F97" s="5"/>
     </row>
-    <row r="98" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A98" s="4">
         <v>6</v>
       </c>
@@ -4389,7 +4392,7 @@
       </c>
       <c r="F98" s="5"/>
     </row>
-    <row r="99" spans="1:6" ht="102" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A99" s="4">
         <v>6</v>
       </c>
@@ -4407,7 +4410,7 @@
       </c>
       <c r="F99" s="5"/>
     </row>
-    <row r="100" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A100" s="4">
         <v>6</v>
       </c>
@@ -4425,7 +4428,7 @@
       </c>
       <c r="F100" s="5"/>
     </row>
-    <row r="101" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A101" s="4">
         <v>6</v>
       </c>
@@ -4443,7 +4446,7 @@
       </c>
       <c r="F101" s="5"/>
     </row>
-    <row r="102" spans="1:6" ht="102" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A102" s="4">
         <v>6</v>
       </c>
@@ -4461,7 +4464,7 @@
       </c>
       <c r="F102" s="5"/>
     </row>
-    <row r="103" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" ht="237.6" x14ac:dyDescent="0.3">
       <c r="A103" s="4">
         <v>7</v>
       </c>
@@ -4479,7 +4482,7 @@
       </c>
       <c r="F103" s="5"/>
     </row>
-    <row r="104" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" ht="237.6" x14ac:dyDescent="0.3">
       <c r="A104" s="4">
         <v>7</v>
       </c>
@@ -4497,7 +4500,7 @@
       </c>
       <c r="F104" s="5"/>
     </row>
-    <row r="105" spans="1:6" ht="318.75" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" ht="330" x14ac:dyDescent="0.3">
       <c r="A105" s="4">
         <v>7</v>
       </c>
@@ -4515,7 +4518,7 @@
       </c>
       <c r="F105" s="5"/>
     </row>
-    <row r="106" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A106" s="4">
         <v>7</v>
       </c>
@@ -4533,7 +4536,7 @@
       </c>
       <c r="F106" s="5"/>
     </row>
-    <row r="107" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A107" s="4">
         <v>7</v>
       </c>
@@ -4551,7 +4554,7 @@
       </c>
       <c r="F107" s="5"/>
     </row>
-    <row r="108" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" ht="303.60000000000002" x14ac:dyDescent="0.3">
       <c r="A108" s="4">
         <v>7</v>
       </c>
@@ -4571,7 +4574,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="109" spans="1:6" ht="267.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" ht="250.8" x14ac:dyDescent="0.3">
       <c r="A109" s="4">
         <v>7</v>
       </c>
@@ -4591,7 +4594,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="110" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A110" s="4">
         <v>7</v>
       </c>
@@ -4611,7 +4614,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="280.5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" ht="290.39999999999998" x14ac:dyDescent="0.3">
       <c r="A111" s="4">
         <v>7</v>
       </c>
@@ -4629,7 +4632,7 @@
       </c>
       <c r="F111" s="5"/>
     </row>
-    <row r="112" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A112" s="4">
         <v>7</v>
       </c>
@@ -4647,7 +4650,7 @@
       </c>
       <c r="F112" s="5"/>
     </row>
-    <row r="113" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A113" s="4">
         <v>7</v>
       </c>
@@ -4665,7 +4668,7 @@
       </c>
       <c r="F113" s="5"/>
     </row>
-    <row r="114" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A114" s="4">
         <v>7</v>
       </c>
@@ -4683,7 +4686,7 @@
       </c>
       <c r="F114" s="5"/>
     </row>
-    <row r="115" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A115" s="4">
         <v>8</v>
       </c>
@@ -4701,7 +4704,7 @@
       </c>
       <c r="F115" s="5"/>
     </row>
-    <row r="116" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A116" s="4">
         <v>8</v>
       </c>
@@ -4719,7 +4722,7 @@
       </c>
       <c r="F116" s="5"/>
     </row>
-    <row r="117" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" ht="198" x14ac:dyDescent="0.3">
       <c r="A117" s="4">
         <v>8</v>
       </c>
@@ -4737,7 +4740,7 @@
       </c>
       <c r="F117" s="5"/>
     </row>
-    <row r="118" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A118" s="4">
         <v>8</v>
       </c>
@@ -4755,7 +4758,7 @@
       </c>
       <c r="F118" s="5"/>
     </row>
-    <row r="119" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" ht="198" x14ac:dyDescent="0.3">
       <c r="A119" s="4">
         <v>8</v>
       </c>
@@ -4773,7 +4776,7 @@
       </c>
       <c r="F119" s="5"/>
     </row>
-    <row r="120" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A120" s="4">
         <v>8</v>
       </c>
@@ -4791,7 +4794,7 @@
       </c>
       <c r="F120" s="5"/>
     </row>
-    <row r="121" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" ht="198" x14ac:dyDescent="0.3">
       <c r="A121" s="4">
         <v>8</v>
       </c>
@@ -4809,7 +4812,7 @@
       </c>
       <c r="F121" s="5"/>
     </row>
-    <row r="122" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" ht="198" x14ac:dyDescent="0.3">
       <c r="A122" s="4">
         <v>8</v>
       </c>
@@ -4827,7 +4830,7 @@
       </c>
       <c r="F122" s="5"/>
     </row>
-    <row r="123" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A123" s="4">
         <v>8</v>
       </c>
@@ -4845,7 +4848,7 @@
       </c>
       <c r="F123" s="5"/>
     </row>
-    <row r="124" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" ht="198" x14ac:dyDescent="0.3">
       <c r="A124" s="4">
         <v>8</v>
       </c>
@@ -4863,7 +4866,7 @@
       </c>
       <c r="F124" s="5"/>
     </row>
-    <row r="125" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A125" s="4">
         <v>8</v>
       </c>
@@ -4881,7 +4884,7 @@
       </c>
       <c r="F125" s="5"/>
     </row>
-    <row r="126" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A126" s="4">
         <v>8</v>
       </c>
@@ -4899,7 +4902,7 @@
       </c>
       <c r="F126" s="5"/>
     </row>
-    <row r="127" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A127" s="4">
         <v>8</v>
       </c>
@@ -4917,7 +4920,7 @@
       </c>
       <c r="F127" s="5"/>
     </row>
-    <row r="128" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A128" s="4">
         <v>8</v>
       </c>
@@ -4935,7 +4938,7 @@
       </c>
       <c r="F128" s="5"/>
     </row>
-    <row r="129" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A129" s="4">
         <v>8</v>
       </c>
@@ -4953,7 +4956,7 @@
       </c>
       <c r="F129" s="5"/>
     </row>
-    <row r="130" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" ht="237.6" x14ac:dyDescent="0.3">
       <c r="A130" s="4">
         <v>8</v>
       </c>
@@ -4971,7 +4974,7 @@
       </c>
       <c r="F130" s="5"/>
     </row>
-    <row r="131" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A131" s="4">
         <v>8</v>
       </c>
@@ -4989,7 +4992,7 @@
       </c>
       <c r="F131" s="5"/>
     </row>
-    <row r="132" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" ht="409.2" x14ac:dyDescent="0.3">
       <c r="A132" s="4">
         <v>8</v>
       </c>
@@ -5007,7 +5010,7 @@
       </c>
       <c r="F132" s="5"/>
     </row>
-    <row r="133" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A133" s="4">
         <v>8</v>
       </c>
@@ -5025,7 +5028,7 @@
       </c>
       <c r="F133" s="5"/>
     </row>
-    <row r="134" spans="1:6" ht="357" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" ht="356.4" x14ac:dyDescent="0.3">
       <c r="A134" s="4">
         <v>8</v>
       </c>
@@ -5043,7 +5046,7 @@
       </c>
       <c r="F134" s="5"/>
     </row>
-    <row r="135" spans="1:6" ht="369.75" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" ht="382.8" x14ac:dyDescent="0.3">
       <c r="A135" s="4">
         <v>8</v>
       </c>
@@ -5063,7 +5066,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="136" spans="1:6" ht="255" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" ht="264" x14ac:dyDescent="0.3">
       <c r="A136" s="4">
         <v>8</v>
       </c>
@@ -5081,7 +5084,7 @@
       </c>
       <c r="F136" s="5"/>
     </row>
-    <row r="137" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A137" s="4">
         <v>8</v>
       </c>
@@ -5099,7 +5102,7 @@
       </c>
       <c r="F137" s="5"/>
     </row>
-    <row r="138" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A138" s="4">
         <v>8</v>
       </c>
@@ -5119,7 +5122,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="139" spans="1:6" ht="280.5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" ht="277.2" x14ac:dyDescent="0.3">
       <c r="A139" s="4">
         <v>8</v>
       </c>
@@ -5137,7 +5140,7 @@
       </c>
       <c r="F139" s="5"/>
     </row>
-    <row r="140" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A140" s="4">
         <v>8</v>
       </c>
@@ -5157,7 +5160,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="141" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A141" s="4">
         <v>8</v>
       </c>
@@ -5177,7 +5180,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="142" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A142" s="4">
         <v>8</v>
       </c>
@@ -5197,7 +5200,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="143" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A143" s="4">
         <v>8</v>
       </c>
@@ -5217,7 +5220,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="144" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A144" s="4">
         <v>9</v>
       </c>
@@ -5235,7 +5238,7 @@
       </c>
       <c r="F144" s="5"/>
     </row>
-    <row r="145" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A145" s="4">
         <v>9</v>
       </c>
@@ -5253,7 +5256,7 @@
       </c>
       <c r="F145" s="5"/>
     </row>
-    <row r="146" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A146" s="4">
         <v>9</v>
       </c>
@@ -5271,7 +5274,7 @@
       </c>
       <c r="F146" s="5"/>
     </row>
-    <row r="147" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A147" s="4">
         <v>9</v>
       </c>
@@ -5289,7 +5292,7 @@
       </c>
       <c r="F147" s="5"/>
     </row>
-    <row r="148" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A148" s="4">
         <v>9</v>
       </c>
@@ -5307,7 +5310,7 @@
       </c>
       <c r="F148" s="5"/>
     </row>
-    <row r="149" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A149" s="4">
         <v>9</v>
       </c>
@@ -5325,7 +5328,7 @@
       </c>
       <c r="F149" s="5"/>
     </row>
-    <row r="150" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A150" s="4">
         <v>9</v>
       </c>
@@ -5343,7 +5346,7 @@
       </c>
       <c r="F150" s="5"/>
     </row>
-    <row r="151" spans="1:6" ht="344.25" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" ht="330" x14ac:dyDescent="0.3">
       <c r="A151" s="4">
         <v>9</v>
       </c>
@@ -5361,7 +5364,7 @@
       </c>
       <c r="F151" s="5"/>
     </row>
-    <row r="152" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A152" s="4">
         <v>9</v>
       </c>
@@ -5379,7 +5382,7 @@
       </c>
       <c r="F152" s="5"/>
     </row>
-    <row r="153" spans="1:6" ht="331.5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" ht="330" x14ac:dyDescent="0.3">
       <c r="A153" s="4">
         <v>9</v>
       </c>
@@ -5397,7 +5400,7 @@
       </c>
       <c r="F153" s="5"/>
     </row>
-    <row r="154" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A154" s="4">
         <v>9</v>
       </c>
@@ -5415,7 +5418,7 @@
       </c>
       <c r="F154" s="5"/>
     </row>
-    <row r="155" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A155" s="4">
         <v>9</v>
       </c>
@@ -5433,7 +5436,7 @@
       </c>
       <c r="F155" s="5"/>
     </row>
-    <row r="156" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A156" s="4">
         <v>9</v>
       </c>
@@ -5451,7 +5454,7 @@
       </c>
       <c r="F156" s="5"/>
     </row>
-    <row r="157" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A157" s="4">
         <v>9</v>
       </c>
@@ -5469,7 +5472,7 @@
       </c>
       <c r="F157" s="5"/>
     </row>
-    <row r="158" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A158" s="4">
         <v>9</v>
       </c>
@@ -5487,7 +5490,7 @@
       </c>
       <c r="F158" s="5"/>
     </row>
-    <row r="159" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A159" s="4">
         <v>9</v>
       </c>
@@ -5505,7 +5508,7 @@
       </c>
       <c r="F159" s="5"/>
     </row>
-    <row r="160" spans="1:6" ht="242.25" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" ht="250.8" x14ac:dyDescent="0.3">
       <c r="A160" s="4">
         <v>9</v>
       </c>
@@ -5523,7 +5526,7 @@
       </c>
       <c r="F160" s="5"/>
     </row>
-    <row r="161" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A161" s="4">
         <v>9</v>
       </c>
@@ -5541,7 +5544,7 @@
       </c>
       <c r="F161" s="5"/>
     </row>
-    <row r="162" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A162" s="4">
         <v>9</v>
       </c>
@@ -5559,7 +5562,7 @@
       </c>
       <c r="F162" s="5"/>
     </row>
-    <row r="163" spans="1:6" ht="293.25" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" ht="303.60000000000002" x14ac:dyDescent="0.3">
       <c r="A163" s="4">
         <v>9</v>
       </c>
@@ -5577,7 +5580,7 @@
       </c>
       <c r="F163" s="5"/>
     </row>
-    <row r="164" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A164" s="4">
         <v>9</v>
       </c>
@@ -5595,7 +5598,7 @@
       </c>
       <c r="F164" s="5"/>
     </row>
-    <row r="165" spans="1:6" ht="408" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" ht="409.2" x14ac:dyDescent="0.3">
       <c r="A165" s="4">
         <v>9</v>
       </c>
@@ -5613,7 +5616,7 @@
       </c>
       <c r="F165" s="5"/>
     </row>
-    <row r="166" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A166" s="4">
         <v>9</v>
       </c>
@@ -5631,7 +5634,7 @@
       </c>
       <c r="F166" s="5"/>
     </row>
-    <row r="167" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A167" s="4">
         <v>9</v>
       </c>
@@ -5649,7 +5652,7 @@
       </c>
       <c r="F167" s="5"/>
     </row>
-    <row r="168" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" ht="198" x14ac:dyDescent="0.3">
       <c r="A168" s="4">
         <v>9</v>
       </c>
@@ -5669,7 +5672,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="169" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A169" s="4">
         <v>9</v>
       </c>
@@ -5687,7 +5690,7 @@
       </c>
       <c r="F169" s="5"/>
     </row>
-    <row r="170" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" ht="237.6" x14ac:dyDescent="0.3">
       <c r="A170" s="4">
         <v>10</v>
       </c>
@@ -5705,7 +5708,7 @@
       </c>
       <c r="F170" s="5"/>
     </row>
-    <row r="171" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" ht="237.6" x14ac:dyDescent="0.3">
       <c r="A171" s="4">
         <v>10</v>
       </c>
@@ -5723,7 +5726,7 @@
       </c>
       <c r="F171" s="5"/>
     </row>
-    <row r="172" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A172" s="4">
         <v>10</v>
       </c>
@@ -5741,7 +5744,7 @@
       </c>
       <c r="F172" s="5"/>
     </row>
-    <row r="173" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A173" s="4">
         <v>10</v>
       </c>
@@ -5759,7 +5762,7 @@
       </c>
       <c r="F173" s="5"/>
     </row>
-    <row r="174" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A174" s="4">
         <v>10</v>
       </c>
@@ -5777,7 +5780,7 @@
       </c>
       <c r="F174" s="5"/>
     </row>
-    <row r="175" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A175" s="4">
         <v>10</v>
       </c>
@@ -5795,7 +5798,7 @@
       </c>
       <c r="F175" s="5"/>
     </row>
-    <row r="176" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A176" s="4">
         <v>10</v>
       </c>
@@ -5813,7 +5816,7 @@
       </c>
       <c r="F176" s="5"/>
     </row>
-    <row r="177" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A177" s="4">
         <v>10</v>
       </c>
@@ -5831,7 +5834,7 @@
       </c>
       <c r="F177" s="5"/>
     </row>
-    <row r="178" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A178" s="4">
         <v>10</v>
       </c>
@@ -5849,7 +5852,7 @@
       </c>
       <c r="F178" s="5"/>
     </row>
-    <row r="179" spans="1:6" ht="255" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:6" ht="264" x14ac:dyDescent="0.3">
       <c r="A179" s="4">
         <v>10</v>
       </c>
@@ -5867,7 +5870,7 @@
       </c>
       <c r="F179" s="5"/>
     </row>
-    <row r="180" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A180" s="4">
         <v>10</v>
       </c>
@@ -5885,7 +5888,7 @@
       </c>
       <c r="F180" s="5"/>
     </row>
-    <row r="181" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A181" s="4">
         <v>10</v>
       </c>
@@ -5903,7 +5906,7 @@
       </c>
       <c r="F181" s="5"/>
     </row>
-    <row r="182" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A182" s="4">
         <v>10</v>
       </c>
@@ -5921,7 +5924,7 @@
       </c>
       <c r="F182" s="5"/>
     </row>
-    <row r="183" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A183" s="4">
         <v>10</v>
       </c>
@@ -5939,7 +5942,7 @@
       </c>
       <c r="F183" s="5"/>
     </row>
-    <row r="184" spans="1:6" ht="395.25" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" ht="396" x14ac:dyDescent="0.3">
       <c r="A184" s="4">
         <v>10</v>
       </c>
@@ -5957,7 +5960,7 @@
       </c>
       <c r="F184" s="5"/>
     </row>
-    <row r="185" spans="1:6" ht="102" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A185" s="4">
         <v>10</v>
       </c>
@@ -5977,7 +5980,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="186" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A186" s="4">
         <v>10</v>
       </c>
@@ -5995,7 +5998,7 @@
       </c>
       <c r="F186" s="6"/>
     </row>
-    <row r="187" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A187" s="4">
         <v>10</v>
       </c>
@@ -6015,7 +6018,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="188" spans="1:6" ht="102" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:6" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A188" s="4">
         <v>10</v>
       </c>
@@ -6033,7 +6036,7 @@
       </c>
       <c r="F188" s="5"/>
     </row>
-    <row r="189" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A189" s="4">
         <v>10</v>
       </c>
@@ -6051,7 +6054,7 @@
       </c>
       <c r="F189" s="5"/>
     </row>
-    <row r="190" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A190" s="4">
         <v>10</v>
       </c>
@@ -6069,7 +6072,7 @@
       </c>
       <c r="F190" s="5"/>
     </row>
-    <row r="191" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A191" s="4">
         <v>10</v>
       </c>
@@ -6087,7 +6090,7 @@
       </c>
       <c r="F191" s="5"/>
     </row>
-    <row r="192" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A192" s="4">
         <v>10</v>
       </c>
@@ -6105,7 +6108,7 @@
       </c>
       <c r="F192" s="5"/>
     </row>
-    <row r="193" spans="1:6" ht="344.25" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:6" ht="356.4" x14ac:dyDescent="0.3">
       <c r="A193" s="4">
         <v>10</v>
       </c>
@@ -6123,10 +6126,16 @@
       </c>
       <c r="F193" s="5"/>
     </row>
-    <row r="194" spans="1:6" ht="204" x14ac:dyDescent="0.25">
-      <c r="A194" s="4"/>
-      <c r="B194" s="4"/>
-      <c r="C194" s="5"/>
+    <row r="194" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
+      <c r="A194" s="4">
+        <v>10</v>
+      </c>
+      <c r="B194" s="4">
+        <v>10.7</v>
+      </c>
+      <c r="C194" s="5" t="s">
+        <v>580</v>
+      </c>
       <c r="D194" s="4" t="s">
         <v>433</v>
       </c>
@@ -6137,7 +6146,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="195" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A195" s="4">
         <v>10</v>
       </c>
@@ -6155,7 +6164,7 @@
       </c>
       <c r="F195" s="6"/>
     </row>
-    <row r="196" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A196" s="4">
         <v>11</v>
       </c>
@@ -6173,7 +6182,7 @@
       </c>
       <c r="F196" s="5"/>
     </row>
-    <row r="197" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:6" ht="211.2" x14ac:dyDescent="0.3">
       <c r="A197" s="4">
         <v>11</v>
       </c>
@@ -6191,7 +6200,7 @@
       </c>
       <c r="F197" s="5"/>
     </row>
-    <row r="198" spans="1:6" ht="344.25" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:6" ht="356.4" x14ac:dyDescent="0.3">
       <c r="A198" s="4">
         <v>11</v>
       </c>
@@ -6209,7 +6218,7 @@
       </c>
       <c r="F198" s="5"/>
     </row>
-    <row r="199" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A199" s="4">
         <v>11</v>
       </c>
@@ -6227,7 +6236,7 @@
       </c>
       <c r="F199" s="5"/>
     </row>
-    <row r="200" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A200" s="4">
         <v>11</v>
       </c>
@@ -6245,7 +6254,7 @@
       </c>
       <c r="F200" s="5"/>
     </row>
-    <row r="201" spans="1:6" ht="357" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:6" ht="356.4" x14ac:dyDescent="0.3">
       <c r="A201" s="4">
         <v>11</v>
       </c>
@@ -6265,7 +6274,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="202" spans="1:6" ht="382.5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:6" ht="356.4" x14ac:dyDescent="0.3">
       <c r="A202" s="4">
         <v>11</v>
       </c>
@@ -6285,7 +6294,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="203" spans="1:6" ht="357" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:6" ht="356.4" x14ac:dyDescent="0.3">
       <c r="A203" s="4">
         <v>11</v>
       </c>
@@ -6303,7 +6312,7 @@
       </c>
       <c r="F203" s="5"/>
     </row>
-    <row r="204" spans="1:6" ht="357" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:6" ht="356.4" x14ac:dyDescent="0.3">
       <c r="A204" s="4">
         <v>11</v>
       </c>
@@ -6321,7 +6330,7 @@
       </c>
       <c r="F204" s="5"/>
     </row>
-    <row r="205" spans="1:6" ht="306" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:6" ht="303.60000000000002" x14ac:dyDescent="0.3">
       <c r="A205" s="4">
         <v>11</v>
       </c>
@@ -6339,7 +6348,7 @@
       </c>
       <c r="F205" s="5"/>
     </row>
-    <row r="206" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A206" s="4">
         <v>11</v>
       </c>
@@ -6357,7 +6366,7 @@
       </c>
       <c r="F206" s="5"/>
     </row>
-    <row r="207" spans="1:6" ht="331.5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:6" ht="330" x14ac:dyDescent="0.3">
       <c r="A207" s="4">
         <v>11</v>
       </c>
@@ -6375,7 +6384,7 @@
       </c>
       <c r="F207" s="5"/>
     </row>
-    <row r="208" spans="1:6" ht="318.75" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:6" ht="303.60000000000002" x14ac:dyDescent="0.3">
       <c r="A208" s="4">
         <v>11</v>
       </c>
@@ -6393,7 +6402,7 @@
       </c>
       <c r="F208" s="5"/>
     </row>
-    <row r="209" spans="1:6" ht="267.75" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:6" ht="264" x14ac:dyDescent="0.3">
       <c r="A209" s="4">
         <v>11</v>
       </c>
@@ -6411,7 +6420,7 @@
       </c>
       <c r="F209" s="5"/>
     </row>
-    <row r="210" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A210" s="4">
         <v>11</v>
       </c>
@@ -6429,7 +6438,7 @@
       </c>
       <c r="F210" s="5"/>
     </row>
-    <row r="211" spans="1:6" ht="242.25" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:6" ht="237.6" x14ac:dyDescent="0.3">
       <c r="A211" s="4">
         <v>11</v>
       </c>
@@ -6447,7 +6456,7 @@
       </c>
       <c r="F211" s="5"/>
     </row>
-    <row r="212" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A212" s="4">
         <v>11</v>
       </c>
@@ -6465,7 +6474,7 @@
       </c>
       <c r="F212" s="5"/>
     </row>
-    <row r="213" spans="1:6" ht="229.5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:6" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A213" s="4">
         <v>11</v>
       </c>
@@ -6483,7 +6492,7 @@
       </c>
       <c r="F213" s="5"/>
     </row>
-    <row r="214" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A214" s="4">
         <v>11</v>
       </c>
@@ -6503,7 +6512,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="215" spans="1:6" ht="280.5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:6" ht="277.2" x14ac:dyDescent="0.3">
       <c r="A215" s="4">
         <v>11</v>
       </c>
@@ -6521,7 +6530,7 @@
       </c>
       <c r="F215" s="5"/>
     </row>
-    <row r="216" spans="1:6" ht="242.25" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:6" ht="250.8" x14ac:dyDescent="0.3">
       <c r="A216" s="4">
         <v>11</v>
       </c>
@@ -6541,7 +6550,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="217" spans="1:6" ht="255" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:6" ht="264" x14ac:dyDescent="0.3">
       <c r="A217" s="4">
         <v>12</v>
       </c>
@@ -6559,7 +6568,7 @@
       </c>
       <c r="F217" s="5"/>
     </row>
-    <row r="218" spans="1:6" ht="255" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:6" ht="264" x14ac:dyDescent="0.3">
       <c r="A218" s="4">
         <v>12</v>
       </c>
@@ -6577,7 +6586,7 @@
       </c>
       <c r="F218" s="5"/>
     </row>
-    <row r="219" spans="1:6" ht="255" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:6" ht="264" x14ac:dyDescent="0.3">
       <c r="A219" s="4">
         <v>12</v>
       </c>
@@ -6595,7 +6604,7 @@
       </c>
       <c r="F219" s="5"/>
     </row>
-    <row r="220" spans="1:6" ht="242.25" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:6" ht="237.6" x14ac:dyDescent="0.3">
       <c r="A220" s="4">
         <v>12</v>
       </c>
@@ -6613,7 +6622,7 @@
       </c>
       <c r="F220" s="5"/>
     </row>
-    <row r="221" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A221" s="4">
         <v>12</v>
       </c>
@@ -6633,7 +6642,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="222" spans="1:6" ht="408" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:6" ht="409.2" x14ac:dyDescent="0.3">
       <c r="A222" s="4">
         <v>12</v>
       </c>
@@ -6651,7 +6660,7 @@
       </c>
       <c r="F222" s="5"/>
     </row>
-    <row r="223" spans="1:6" ht="408" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A223" s="4">
         <v>12</v>
       </c>
@@ -6671,7 +6680,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="224" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A224" s="4">
         <v>12</v>
       </c>
@@ -6691,7 +6700,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="225" spans="1:6" ht="267.75" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:6" ht="277.2" x14ac:dyDescent="0.3">
       <c r="A225" s="4">
         <v>12</v>
       </c>
@@ -6709,7 +6718,7 @@
       </c>
       <c r="F225" s="5"/>
     </row>
-    <row r="226" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A226" s="4">
         <v>12</v>
       </c>
@@ -6727,7 +6736,7 @@
       </c>
       <c r="F226" s="5"/>
     </row>
-    <row r="227" spans="1:6" ht="318.75" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:6" ht="330" x14ac:dyDescent="0.3">
       <c r="A227" s="4">
         <v>12</v>
       </c>
@@ -6745,7 +6754,7 @@
       </c>
       <c r="F227" s="5"/>
     </row>
-    <row r="228" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A228" s="4">
         <v>12</v>
       </c>
@@ -6763,7 +6772,7 @@
       </c>
       <c r="F228" s="5"/>
     </row>
-    <row r="229" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A229" s="4">
         <v>12</v>
       </c>
@@ -6781,7 +6790,7 @@
       </c>
       <c r="F229" s="5"/>
     </row>
-    <row r="230" spans="1:6" ht="204" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:6" ht="198" x14ac:dyDescent="0.3">
       <c r="A230" s="4">
         <v>12</v>
       </c>
@@ -6801,7 +6810,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="231" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A231" s="4">
         <v>12</v>
       </c>
@@ -6821,7 +6830,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="232" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A232" s="4">
         <v>12</v>
       </c>
@@ -6839,7 +6848,7 @@
       </c>
       <c r="F232" s="5"/>
     </row>
-    <row r="233" spans="1:6" ht="255" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:6" ht="250.8" x14ac:dyDescent="0.3">
       <c r="A233" s="4">
         <v>12</v>
       </c>
@@ -6859,7 +6868,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="234" spans="1:6" ht="255" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:6" ht="250.8" x14ac:dyDescent="0.3">
       <c r="A234" s="4">
         <v>12</v>
       </c>
@@ -6877,7 +6886,7 @@
       </c>
       <c r="F234" s="5"/>
     </row>
-    <row r="235" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A235" s="4">
         <v>12</v>
       </c>
@@ -6897,7 +6906,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="236" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A236" s="4">
         <v>12</v>
       </c>
@@ -6917,7 +6926,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="237" spans="1:6" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:6" ht="145.19999999999999" x14ac:dyDescent="0.3">
       <c r="A237" s="4">
         <v>12</v>
       </c>
@@ -6935,7 +6944,7 @@
       </c>
       <c r="F237" s="5"/>
     </row>
-    <row r="238" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A238" s="4">
         <v>12</v>
       </c>
@@ -6953,7 +6962,7 @@
       </c>
       <c r="F238" s="5"/>
     </row>
-    <row r="239" spans="1:6" ht="408" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A239" s="4">
         <v>12</v>
       </c>
@@ -6971,7 +6980,7 @@
       </c>
       <c r="F239" s="5"/>
     </row>
-    <row r="240" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A240" s="4">
         <v>12</v>
       </c>
@@ -6989,7 +6998,7 @@
       </c>
       <c r="F240" s="5"/>
     </row>
-    <row r="241" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A241" s="4">
         <v>12</v>
       </c>
@@ -7007,7 +7016,7 @@
       </c>
       <c r="F241" s="5"/>
     </row>
-    <row r="242" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A242" s="4">
         <v>12</v>
       </c>
@@ -7025,7 +7034,7 @@
       </c>
       <c r="F242" s="5"/>
     </row>
-    <row r="243" spans="1:6" ht="267.75" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:6" ht="264" x14ac:dyDescent="0.3">
       <c r="A243" s="4">
         <v>12</v>
       </c>
@@ -7043,7 +7052,7 @@
       </c>
       <c r="F243" s="5"/>
     </row>
-    <row r="244" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A244" s="4">
         <v>12</v>
       </c>
@@ -7061,7 +7070,7 @@
       </c>
       <c r="F244" s="5"/>
     </row>
-    <row r="245" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A245" s="4">
         <v>12</v>
       </c>
@@ -7079,7 +7088,7 @@
       </c>
       <c r="F245" s="5"/>
     </row>
-    <row r="246" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A246" s="4">
         <v>12</v>
       </c>
@@ -7097,7 +7106,7 @@
       </c>
       <c r="F246" s="5"/>
     </row>
-    <row r="247" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A247" s="4">
         <v>12</v>
       </c>
@@ -7115,7 +7124,7 @@
       </c>
       <c r="F247" s="5"/>
     </row>
-    <row r="248" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A248" s="4">
         <v>12</v>
       </c>
@@ -7133,7 +7142,7 @@
       </c>
       <c r="F248" s="5"/>
     </row>
-    <row r="249" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A249" s="4">
         <v>12</v>
       </c>
@@ -7151,7 +7160,7 @@
       </c>
       <c r="F249" s="5"/>
     </row>
-    <row r="250" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A250" s="4">
         <v>12</v>
       </c>
@@ -7171,7 +7180,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="251" spans="1:6" ht="331.5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:6" ht="330" x14ac:dyDescent="0.3">
       <c r="A251" s="4">
         <v>12</v>
       </c>
@@ -7189,7 +7198,7 @@
       </c>
       <c r="F251" s="6"/>
     </row>
-    <row r="252" spans="1:6" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A252" s="4">
         <v>12</v>
       </c>
@@ -7209,7 +7218,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="253" spans="1:6" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:6" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A253" s="4">
         <v>12</v>
       </c>
@@ -7227,7 +7236,7 @@
       </c>
       <c r="F253" s="5"/>
     </row>
-    <row r="254" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A254" s="4">
         <v>12</v>
       </c>
@@ -7247,7 +7256,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="255" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A255" s="4" t="s">
         <v>571</v>
       </c>
@@ -7265,7 +7274,7 @@
       </c>
       <c r="F255" s="5"/>
     </row>
-    <row r="256" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A256" s="4" t="s">
         <v>571</v>
       </c>
@@ -7283,7 +7292,7 @@
       </c>
       <c r="F256" s="5"/>
     </row>
-    <row r="257" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:6" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A257" s="4" t="s">
         <v>571</v>
       </c>

</xml_diff>